<commit_message>
Release v0.1.1: add LLM fallback and fix generated Excel issues
</commit_message>
<xml_diff>
--- a/template/Test Cases.xlsx
+++ b/template/Test Cases.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D_store\OneDrive - Onrique\Documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1442CF6-6CB9-4CBF-9A83-5DEA7FF9F2E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="583"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="583" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision History" sheetId="6" r:id="rId1"/>
@@ -18,7 +24,20 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Cases'!$6:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Test Results - 1'!$8:$9</definedName>
   </definedNames>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -217,11 +236,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -478,7 +497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -571,29 +590,19 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -628,11 +637,14 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 2" xfId="1"/>
+    <cellStyle name="Normal 2 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -672,7 +684,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -704,9 +716,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -744,7 +756,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -778,6 +790,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -812,9 +825,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -987,42 +1001,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="19.453125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="19.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.08984375" customWidth="1"/>
-    <col min="2" max="2" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="15" thickBot="1">
+    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="43" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
@@ -1036,17 +1050,17 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="48" t="s">
         <v>62</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="48" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1060,23 +1074,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.36328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.36328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="34.26953125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="39" style="8" customWidth="1"/>
-    <col min="6" max="6" width="8.984375E-2" customWidth="1"/>
+    <col min="6" max="6" width="0.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>18</v>
       </c>
@@ -1090,7 +1104,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28">
+    <row r="4" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>21</v>
       </c>
@@ -1104,7 +1118,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>5</v>
       </c>
@@ -1114,293 +1128,258 @@
       <c r="C5" s="30"/>
       <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="1:4" s="1" customFormat="1">
-      <c r="A6" s="45" t="s">
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-    </row>
-    <row r="7" spans="1:4" s="3" customFormat="1">
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+    </row>
+    <row r="7" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="37" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="43.5" customHeight="1">
-      <c r="A8" s="39">
+    <row r="8" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35">
         <v>1</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="39" customHeight="1">
-      <c r="A9" s="39">
+    <row r="9" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="35">
         <v>2</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="32.5" customHeight="1">
-      <c r="A10" s="39">
+    <row r="10" spans="1:4" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="35">
         <v>3</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="34" customHeight="1">
-      <c r="A11" s="39">
+    <row r="11" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="35">
         <v>4</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="29">
-      <c r="A12" s="39">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="35">
         <v>5</v>
       </c>
-      <c r="B12" s="42" t="s">
+      <c r="B12" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="41" customHeight="1">
-      <c r="A13" s="39">
+    <row r="13" spans="1:4" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="35">
         <v>6</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="36.5" customHeight="1">
-      <c r="A14" s="39">
+    <row r="14" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="35">
         <v>7</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C14" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="39.5" customHeight="1">
-      <c r="A15" s="39">
+    <row r="15" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="35">
         <v>8</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="34.5" customHeight="1">
-      <c r="A16" s="39">
+    <row r="16" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="35">
         <v>9</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="33.5" customHeight="1">
-      <c r="A17" s="39">
+    <row r="17" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="35">
         <v>10</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C17" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="40" t="s">
+      <c r="D17" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="34" customHeight="1">
-      <c r="A18" s="39">
+    <row r="18" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="35">
         <v>11</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="C18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="32" customHeight="1">
-      <c r="A19" s="39">
+    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="35">
         <v>12</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="29">
-      <c r="A20" s="39">
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="35">
         <v>13</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="34"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="34"/>
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="37"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="34"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="34"/>
-      <c r="B28" s="36"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="34"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="35"/>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="37"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="35"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="37"/>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="33"/>
+      <c r="D21" s="34"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="33"/>
+      <c r="D22" s="34"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="33"/>
+      <c r="D23" s="34"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="33"/>
+      <c r="D24" s="34"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="33"/>
+      <c r="D25" s="34"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="33"/>
+      <c r="D26" s="34"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="33"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="33"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="33"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Unit Test, Integration Test"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1417,26 +1396,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="69.08984375" style="16" customWidth="1"/>
-    <col min="3" max="3" width="14.08984375" style="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.140625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1">
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="27">
+    <row r="3" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1451,7 +1430,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="27">
+    <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>5</v>
       </c>
@@ -1459,10 +1438,10 @@
         <f>IF(ISBLANK('Test Cases'!B5)," ",'Test Cases'!B5)</f>
         <v>Unit Test</v>
       </c>
-      <c r="C4" s="47"/>
-      <c r="D4" s="48"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="C4" s="43"/>
+      <c r="D4" s="44"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>7</v>
       </c>
@@ -1472,11 +1451,11 @@
       <c r="C5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="33">
+      <c r="D5" s="32">
         <v>46036</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>11</v>
       </c>
@@ -1486,7 +1465,7 @@
       <c r="C6" s="22"/>
       <c r="D6" s="12"/>
     </row>
-    <row r="7" spans="1:4" ht="27">
+    <row r="7" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>9</v>
       </c>
@@ -1496,19 +1475,19 @@
       <c r="C7" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="32">
         <v>46036</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A8" s="49" t="s">
+    <row r="8" spans="1:4" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="51"/>
-    </row>
-    <row r="9" spans="1:4" s="3" customFormat="1">
+      <c r="B8" s="46"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="47"/>
+    </row>
+    <row r="9" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>14</v>
       </c>
@@ -1522,7 +1501,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="24">
         <f>IF(ISBLANK('Test Cases'!A8)," ",'Test Cases'!A8)</f>
         <v>1</v>
@@ -1538,7 +1517,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="20" customHeight="1">
+    <row r="11" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
         <f>IF(ISBLANK('Test Cases'!A9)," ",'Test Cases'!A9)</f>
         <v>2</v>
@@ -1554,7 +1533,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
         <f>IF(ISBLANK('Test Cases'!A10)," ",'Test Cases'!A10)</f>
         <v>3</v>
@@ -1570,7 +1549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <f>IF(ISBLANK('Test Cases'!A11)," ",'Test Cases'!A11)</f>
         <v>4</v>
@@ -1586,7 +1565,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5" customHeight="1">
+    <row r="14" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <f>IF(ISBLANK('Test Cases'!A12)," ",'Test Cases'!A12)</f>
         <v>5</v>
@@ -1602,7 +1581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>6</v>
       </c>
@@ -1617,7 +1596,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="24">
         <v>7</v>
       </c>
@@ -1632,7 +1611,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="24">
         <v>8</v>
       </c>
@@ -1647,7 +1626,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="24">
         <v>9</v>
       </c>
@@ -1662,7 +1641,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="24">
         <v>10</v>
       </c>
@@ -1677,7 +1656,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="24">
         <v>11</v>
       </c>
@@ -1692,7 +1671,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="24">
         <f>IF(ISBLANK('Test Cases'!A19)," ",'Test Cases'!A19)</f>
         <v>12</v>
@@ -1708,7 +1687,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="24">
         <f>IF(ISBLANK('Test Cases'!A20)," ",'Test Cases'!A20)</f>
         <v>13</v>
@@ -1724,7 +1703,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A21)," ",'Test Cases'!A21)</f>
         <v xml:space="preserve"> </v>
@@ -1736,7 +1715,7 @@
       <c r="C23" s="5"/>
       <c r="D23" s="20"/>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A22)," ",'Test Cases'!A22)</f>
         <v xml:space="preserve"> </v>
@@ -1748,7 +1727,7 @@
       <c r="C24" s="5"/>
       <c r="D24" s="20"/>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A23)," ",'Test Cases'!A23)</f>
         <v xml:space="preserve"> </v>
@@ -1760,7 +1739,7 @@
       <c r="C25" s="5"/>
       <c r="D25" s="20"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A24)," ",'Test Cases'!A24)</f>
         <v xml:space="preserve"> </v>
@@ -1772,7 +1751,7 @@
       <c r="C26" s="5"/>
       <c r="D26" s="20"/>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A25)," ",'Test Cases'!A25)</f>
         <v xml:space="preserve"> </v>
@@ -1784,7 +1763,7 @@
       <c r="C27" s="5"/>
       <c r="D27" s="20"/>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A26)," ",'Test Cases'!A26)</f>
         <v xml:space="preserve"> </v>
@@ -1796,7 +1775,7 @@
       <c r="C28" s="5"/>
       <c r="D28" s="20"/>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A27)," ",'Test Cases'!A27)</f>
         <v xml:space="preserve"> </v>
@@ -1808,7 +1787,7 @@
       <c r="C29" s="5"/>
       <c r="D29" s="20"/>
     </row>
-    <row r="30" spans="1:4" ht="15" thickBot="1">
+    <row r="30" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A28)," ",'Test Cases'!A28)</f>
         <v xml:space="preserve"> </v>
@@ -1827,7 +1806,7 @@
     <mergeCell ref="A8:D8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:C30">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:C30" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1840,15 +1819,43 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="5582bb76-1028-4cef-bff8-b84262c5def4" xsi:nil="true"/>
+    <SharedWithUsers xmlns="5582bb76-1028-4cef-bff8-b84262c5def4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BC16F0243930894FBCA21367DF921436" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7d8957b3979d20c20ccc68492b27cd54">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xmlns:ns3="5582bb76-1028-4cef-bff8-b84262c5def4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="404643c56d14aa05f81c1010c52eb386" ns2:_="" ns3:_="">
     <xsd:import namespace="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
@@ -2091,35 +2098,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6A956E9-B18A-45E0-9BE9-125E6EE2068A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
+    <ds:schemaRef ds:uri="5582bb76-1028-4cef-bff8-b84262c5def4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="5582bb76-1028-4cef-bff8-b84262c5def4" xsi:nil="true"/>
-    <SharedWithUsers xmlns="5582bb76-1028-4cef-bff8-b84262c5def4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F54B70-225C-4B04-9A1C-FBA4B4548E82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30DF7585-1C21-45DA-AAF5-8352C9C706BD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2136,23 +2134,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F54B70-225C-4B04-9A1C-FBA4B4548E82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6A956E9-B18A-45E0-9BE9-125E6EE2068A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
-    <ds:schemaRef ds:uri="5582bb76-1028-4cef-bff8-b84262c5def4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Release v0.1.1: add LLM fallback and fix generated Excel issues (#13)
- Add model fallbacks
- Fix date format issue (for this change in template also)
- In TestCase B4 → Ticket ID issue.
</commit_message>
<xml_diff>
--- a/template/Test Cases.xlsx
+++ b/template/Test Cases.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D_store\OneDrive - Onrique\Documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1442CF6-6CB9-4CBF-9A83-5DEA7FF9F2E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="583"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="583" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision History" sheetId="6" r:id="rId1"/>
@@ -18,7 +24,20 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Cases'!$6:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Test Results - 1'!$8:$9</definedName>
   </definedNames>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -217,11 +236,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -478,7 +497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -571,29 +590,19 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -628,11 +637,14 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 2" xfId="1"/>
+    <cellStyle name="Normal 2 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -672,7 +684,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -704,9 +716,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -744,7 +756,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -778,6 +790,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -812,9 +825,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -987,42 +1001,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="19.453125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="19.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.08984375" customWidth="1"/>
-    <col min="2" max="2" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="15" thickBot="1">
+    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="43" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
@@ -1036,17 +1050,17 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="48" t="s">
         <v>62</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="48" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1060,23 +1074,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.36328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.36328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="34.26953125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="39" style="8" customWidth="1"/>
-    <col min="6" max="6" width="8.984375E-2" customWidth="1"/>
+    <col min="6" max="6" width="0.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>18</v>
       </c>
@@ -1090,7 +1104,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28">
+    <row r="4" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>21</v>
       </c>
@@ -1104,7 +1118,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>5</v>
       </c>
@@ -1114,293 +1128,258 @@
       <c r="C5" s="30"/>
       <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="1:4" s="1" customFormat="1">
-      <c r="A6" s="45" t="s">
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-    </row>
-    <row r="7" spans="1:4" s="3" customFormat="1">
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+    </row>
+    <row r="7" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="37" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="43.5" customHeight="1">
-      <c r="A8" s="39">
+    <row r="8" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35">
         <v>1</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="39" customHeight="1">
-      <c r="A9" s="39">
+    <row r="9" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="35">
         <v>2</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="32.5" customHeight="1">
-      <c r="A10" s="39">
+    <row r="10" spans="1:4" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="35">
         <v>3</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="34" customHeight="1">
-      <c r="A11" s="39">
+    <row r="11" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="35">
         <v>4</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="29">
-      <c r="A12" s="39">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="35">
         <v>5</v>
       </c>
-      <c r="B12" s="42" t="s">
+      <c r="B12" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="41" customHeight="1">
-      <c r="A13" s="39">
+    <row r="13" spans="1:4" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="35">
         <v>6</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="36.5" customHeight="1">
-      <c r="A14" s="39">
+    <row r="14" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="35">
         <v>7</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C14" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="39.5" customHeight="1">
-      <c r="A15" s="39">
+    <row r="15" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="35">
         <v>8</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="34.5" customHeight="1">
-      <c r="A16" s="39">
+    <row r="16" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="35">
         <v>9</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="33.5" customHeight="1">
-      <c r="A17" s="39">
+    <row r="17" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="35">
         <v>10</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C17" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="40" t="s">
+      <c r="D17" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="34" customHeight="1">
-      <c r="A18" s="39">
+    <row r="18" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="35">
         <v>11</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="C18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="32" customHeight="1">
-      <c r="A19" s="39">
+    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="35">
         <v>12</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="29">
-      <c r="A20" s="39">
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="35">
         <v>13</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="34"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="34"/>
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="37"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="34"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="34"/>
-      <c r="B28" s="36"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="34"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="35"/>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="37"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="35"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="37"/>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="33"/>
+      <c r="D21" s="34"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="33"/>
+      <c r="D22" s="34"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="33"/>
+      <c r="D23" s="34"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="33"/>
+      <c r="D24" s="34"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="33"/>
+      <c r="D25" s="34"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="33"/>
+      <c r="D26" s="34"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="33"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="33"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="33"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Unit Test, Integration Test"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1417,26 +1396,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="69.08984375" style="16" customWidth="1"/>
-    <col min="3" max="3" width="14.08984375" style="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.140625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1">
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="27">
+    <row r="3" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1451,7 +1430,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="27">
+    <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>5</v>
       </c>
@@ -1459,10 +1438,10 @@
         <f>IF(ISBLANK('Test Cases'!B5)," ",'Test Cases'!B5)</f>
         <v>Unit Test</v>
       </c>
-      <c r="C4" s="47"/>
-      <c r="D4" s="48"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="C4" s="43"/>
+      <c r="D4" s="44"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>7</v>
       </c>
@@ -1472,11 +1451,11 @@
       <c r="C5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="33">
+      <c r="D5" s="32">
         <v>46036</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>11</v>
       </c>
@@ -1486,7 +1465,7 @@
       <c r="C6" s="22"/>
       <c r="D6" s="12"/>
     </row>
-    <row r="7" spans="1:4" ht="27">
+    <row r="7" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>9</v>
       </c>
@@ -1496,19 +1475,19 @@
       <c r="C7" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="32">
         <v>46036</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A8" s="49" t="s">
+    <row r="8" spans="1:4" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="51"/>
-    </row>
-    <row r="9" spans="1:4" s="3" customFormat="1">
+      <c r="B8" s="46"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="47"/>
+    </row>
+    <row r="9" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>14</v>
       </c>
@@ -1522,7 +1501,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="24">
         <f>IF(ISBLANK('Test Cases'!A8)," ",'Test Cases'!A8)</f>
         <v>1</v>
@@ -1538,7 +1517,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="20" customHeight="1">
+    <row r="11" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
         <f>IF(ISBLANK('Test Cases'!A9)," ",'Test Cases'!A9)</f>
         <v>2</v>
@@ -1554,7 +1533,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
         <f>IF(ISBLANK('Test Cases'!A10)," ",'Test Cases'!A10)</f>
         <v>3</v>
@@ -1570,7 +1549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <f>IF(ISBLANK('Test Cases'!A11)," ",'Test Cases'!A11)</f>
         <v>4</v>
@@ -1586,7 +1565,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5" customHeight="1">
+    <row r="14" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <f>IF(ISBLANK('Test Cases'!A12)," ",'Test Cases'!A12)</f>
         <v>5</v>
@@ -1602,7 +1581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>6</v>
       </c>
@@ -1617,7 +1596,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="24">
         <v>7</v>
       </c>
@@ -1632,7 +1611,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="24">
         <v>8</v>
       </c>
@@ -1647,7 +1626,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="24">
         <v>9</v>
       </c>
@@ -1662,7 +1641,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="24">
         <v>10</v>
       </c>
@@ -1677,7 +1656,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="24">
         <v>11</v>
       </c>
@@ -1692,7 +1671,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="24">
         <f>IF(ISBLANK('Test Cases'!A19)," ",'Test Cases'!A19)</f>
         <v>12</v>
@@ -1708,7 +1687,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="24">
         <f>IF(ISBLANK('Test Cases'!A20)," ",'Test Cases'!A20)</f>
         <v>13</v>
@@ -1724,7 +1703,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A21)," ",'Test Cases'!A21)</f>
         <v xml:space="preserve"> </v>
@@ -1736,7 +1715,7 @@
       <c r="C23" s="5"/>
       <c r="D23" s="20"/>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A22)," ",'Test Cases'!A22)</f>
         <v xml:space="preserve"> </v>
@@ -1748,7 +1727,7 @@
       <c r="C24" s="5"/>
       <c r="D24" s="20"/>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A23)," ",'Test Cases'!A23)</f>
         <v xml:space="preserve"> </v>
@@ -1760,7 +1739,7 @@
       <c r="C25" s="5"/>
       <c r="D25" s="20"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A24)," ",'Test Cases'!A24)</f>
         <v xml:space="preserve"> </v>
@@ -1772,7 +1751,7 @@
       <c r="C26" s="5"/>
       <c r="D26" s="20"/>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A25)," ",'Test Cases'!A25)</f>
         <v xml:space="preserve"> </v>
@@ -1784,7 +1763,7 @@
       <c r="C27" s="5"/>
       <c r="D27" s="20"/>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A26)," ",'Test Cases'!A26)</f>
         <v xml:space="preserve"> </v>
@@ -1796,7 +1775,7 @@
       <c r="C28" s="5"/>
       <c r="D28" s="20"/>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A27)," ",'Test Cases'!A27)</f>
         <v xml:space="preserve"> </v>
@@ -1808,7 +1787,7 @@
       <c r="C29" s="5"/>
       <c r="D29" s="20"/>
     </row>
-    <row r="30" spans="1:4" ht="15" thickBot="1">
+    <row r="30" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="24" t="str">
         <f>IF(ISBLANK('Test Cases'!A28)," ",'Test Cases'!A28)</f>
         <v xml:space="preserve"> </v>
@@ -1827,7 +1806,7 @@
     <mergeCell ref="A8:D8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:C30">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:C30" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1840,15 +1819,43 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="5582bb76-1028-4cef-bff8-b84262c5def4" xsi:nil="true"/>
+    <SharedWithUsers xmlns="5582bb76-1028-4cef-bff8-b84262c5def4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BC16F0243930894FBCA21367DF921436" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7d8957b3979d20c20ccc68492b27cd54">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xmlns:ns3="5582bb76-1028-4cef-bff8-b84262c5def4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="404643c56d14aa05f81c1010c52eb386" ns2:_="" ns3:_="">
     <xsd:import namespace="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
@@ -2091,35 +2098,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6A956E9-B18A-45E0-9BE9-125E6EE2068A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
+    <ds:schemaRef ds:uri="5582bb76-1028-4cef-bff8-b84262c5def4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="5582bb76-1028-4cef-bff8-b84262c5def4" xsi:nil="true"/>
-    <SharedWithUsers xmlns="5582bb76-1028-4cef-bff8-b84262c5def4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="6afaaed4-fcad-4e10-9871-7656e03f1fe0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F54B70-225C-4B04-9A1C-FBA4B4548E82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30DF7585-1C21-45DA-AAF5-8352C9C706BD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2136,23 +2134,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F54B70-225C-4B04-9A1C-FBA4B4548E82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6A956E9-B18A-45E0-9BE9-125E6EE2068A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6afaaed4-fcad-4e10-9871-7656e03f1fe0"/>
-    <ds:schemaRef ds:uri="5582bb76-1028-4cef-bff8-b84262c5def4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>